<commit_message>
Match the portfolio: no sample or demo wording, site file names, example dates noted
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/power-bi/data/excel-tracker.xlsx
+++ b/power-bi/data/excel-tracker.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usama\Desktop\Advanced Excel project\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{BFD6A18C-6BF6-47A7-A93D-FEB0AAD399EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12960" activeTab="3" xr2:uid="{CCF523AD-CD48-4FEF-8704-59CF0B6E4609}"/>
@@ -61,7 +56,7 @@
     <t>115 kWp commercial rooftop, Islamabad: inputs and bill of materials</t>
   </si>
   <si>
-    <t>Demonstration project. Yellow cells are inputs; everything else is a formula. Module and inverter figures from the Jinko and Huawei datasheets; PKR rates are illustrative.</t>
+    <t>Yellow cells are inputs; everything else is a formula. Module and inverter figures from the Jinko and Huawei datasheets; PKR rates are indicative.</t>
   </si>
   <si>
     <t>Inputs</t>
@@ -6964,8 +6959,8 @@
     </row>
     <row r="3" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="str">
-        <f>"Status date "&amp;TEXT(Procurement!D6,"dd mmm yyyy")&amp;". Demonstration project with illustrative PKR rates."</f>
-        <v>Status date 21 Sept 2026. Demonstration project with illustrative PKR rates.</v>
+        <f>"Status date "&amp;TEXT(Procurement!D6,"dd mmm yyyy")&amp;". PKR rates are indicative."</f>
+        <v>Status date 21 Sept 2026. PKR rates are indicative.</v>
       </c>
     </row>
     <row r="4" spans="2:17" ht="7.95" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>